<commit_message>
upd naam algoritme checker
</commit_message>
<xml_diff>
--- a/excel-to-ical/voorbeeld rooster/test arjan.xlsx
+++ b/excel-to-ical/voorbeeld rooster/test arjan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sammani/Desktop/Development/AMA app/excel-to-ical/voorbeeld rooster/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39AEAC62-F029-3A42-82DB-70E629FC6E20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85C644A0-C499-C140-9DB4-73BD178CF68D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="800" windowWidth="28800" windowHeight="12300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -207,222 +207,7 @@
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
     <cellStyle name="Standaard 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
-  <dxfs count="26">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <font>
         <b/>
@@ -756,7 +541,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.83203125" customWidth="1"/>
@@ -780,49 +565,53 @@
       <c r="H1" s="5"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B2" s="6">
-        <v>46039</v>
+      <c r="B2" s="6"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B3" s="6">
+        <v>46040</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>3</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D3" t="s">
         <v>0</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E3" t="s">
         <v>1</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F3" t="s">
         <v>2</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G3" t="s">
         <v>4</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B1">
-    <cfRule type="cellIs" dxfId="25" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
       <formula>TODAY()</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="6" operator="lessThan">
+    <cfRule type="cellIs" dxfId="4" priority="6" operator="lessThan">
       <formula>TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1">
-    <cfRule type="cellIs" dxfId="23" priority="137" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="137" operator="equal">
       <formula>"GEANNULEERD"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="138" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="138" operator="equal">
       <formula>"TE PLANNEN"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="139" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="139" operator="equal">
       <formula>"IN BEHANDELING"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="140" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="140" operator="equal">
       <formula>"BEVESTIGD"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>